<commit_message>
Risk-scene renderer: the demo sheet rendered, three dashboards
The demo row, the same row at night (look only: the same contact) and at
90 km/h (motion: the barrier instead), and a roundabout row that cannot be
drawn yet. compose clips a long card heading to the card.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S5ny2rhY6EfqDq7ZohuWRt
</commit_message>
<xml_diff>
--- a/assurance/sim/render-tool/examples/demo.xlsx
+++ b/assurance/sim/render-tool/examples/demo.xlsx
@@ -1121,7 +1121,12 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>exported, not rendered (--no-render)</t>
+          <t>drawn (purchased mesh)</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>row-f-01-m03-os-01-w02.jpg</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1236,7 +1241,12 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>exported, not rendered (--no-render)</t>
+          <t>drawn (purchased mesh)</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>row-f-01-m03-os-01-w02-at-night.jpg</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1354,7 +1364,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>exported, not rendered (--no-render)</t>
+          <t>drawn (purchased mesh)</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>row-f-01-m03-os-01-w02-at-90-km-h.jpg</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1463,6 +1478,11 @@
       <formula1>=Lists!$K$2:$K$65</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T6" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>